<commit_message>
Segmentation decks: animations, slide timings and desk research
- Every slide is animated with no clicks (After Previous): title and line,
  subtitle, then the table, chart or text, then the notes.
- Each slide advances by itself (10 to 35 s, about 4 minutes in all).
- New "Other Research" slide and Research sheet with sources and links.
- "Why" slide now cites the research.
- finish_deck.py gains --advance and a Wipe From Top effect; deck_kit
  records the animation plan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WToQxHdrdWhM7bKqXvUa59
</commit_message>
<xml_diff>
--- a/segmentation/Segmentation_Matrix.xlsx
+++ b/segmentation/Segmentation_Matrix.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Segmentation Matrix" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attractiveness" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +83,14 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -122,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -159,6 +168,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
@@ -1534,4 +1546,212 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="21" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DESK RESEARCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Other research that backs up the Google Trends findings and the scores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Trends data: Google Trends, Nigeria, past 12 months (28 September 2025 to 28 September 2026). Web sources found on 8 October 2026; figures as the sources report them. Click a link to open the source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Finding</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Segment it supports</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>The CAC confirmed a cyber breach of its systems in April 2026, and the data protection commission (NDPC) opened an investigation.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Cybersecurity</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>AllAfrica, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>allafrica.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Nigeria had only about 8,352 cybersecurity professionals in 2023, against 57,269 in South Africa.</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Cybersecurity</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>ISC2 figures, reported by CompTIA</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>comptia.org</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Nigerian organisations faced about 4,388 cyber attacks a week in early 2025, 47% more than a year before.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Cybersecurity</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Check Point, reported by BusinessDay</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>businessday.ng</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>About 14 million Nigerian small businesses used Facebook, Instagram and WhatsApp in 2025.</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Digital marketing</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Public First report for Meta, reported by IT Edge News</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>itedgenews.africa</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>The government's 3MTT programme aims to train three million tech talents by 2027, so demand for tech skills is growing, but free training also competes.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>All five</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Federal Ministry of Communications, Innovation and Digital Economy</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>3mtt.nitda.gov.ng</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId5"/>
+  </hyperlinks>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>